<commit_message>
Change 3B reference to False
</commit_message>
<xml_diff>
--- a/output/tables/tab_3A_weights.xlsx
+++ b/output/tables/tab_3A_weights.xlsx
@@ -488,10 +488,10 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.06381776251846305</v>
+        <v>0.06381776251846315</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.1067618290499486</v>
+        <v>0.1067618290499489</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0.02228938330568139</v>
@@ -509,13 +509,13 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.1947591593607026</v>
+        <v>0.194759159360703</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.09053460558371441</v>
+        <v>0.09053460558371493</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.02912158888875273</v>
+        <v>0.02912158888875272</v>
       </c>
     </row>
     <row r="4">
@@ -530,7 +530,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>-0.05142746702816062</v>
+        <v>-0.05142746702816055</v>
       </c>
       <c r="D4" s="4" t="n">
         <v>0</v>
@@ -551,13 +551,13 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-0.01806947171145539</v>
+        <v>-0.01806947171145564</v>
       </c>
       <c r="D5" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.02107967464818333</v>
+        <v>0.02107967464818332</v>
       </c>
     </row>
     <row r="6">
@@ -572,13 +572,13 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.0006714307443167332</v>
+        <v>0.0006714307443165005</v>
       </c>
       <c r="D6" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>0.01449736814887323</v>
+        <v>0.01449736814887322</v>
       </c>
     </row>
     <row r="7">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-0.005151232639393402</v>
+        <v>-0.005151232639393697</v>
       </c>
       <c r="D7" s="4" t="n">
         <v>0</v>
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.01319967294020989</v>
+        <v>0.01319967294020996</v>
       </c>
       <c r="D8" s="4" t="n">
         <v>0</v>
@@ -635,10 +635,10 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>0.4127534433949248</v>
+        <v>0.4127534433949251</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.07724415341713295</v>
+        <v>0.07724415341713207</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0.0268553736347916</v>
@@ -656,10 +656,10 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.2115424508138969</v>
+        <v>0.2115424508138975</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>0.122812677355998</v>
+        <v>0.1228126773559982</v>
       </c>
       <c r="E10" s="3" t="n">
         <v>0.02745905454959906</v>
@@ -677,13 +677,13 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.02257890968362071</v>
+        <v>0.02257890968362105</v>
       </c>
       <c r="D11" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>0.02001709413173895</v>
+        <v>0.02001709413173894</v>
       </c>
     </row>
     <row r="12">
@@ -698,7 +698,7 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>-0.04921506446718911</v>
+        <v>-0.04921506446718899</v>
       </c>
       <c r="D12" s="4" t="n">
         <v>0</v>
@@ -719,10 +719,10 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>0.2519863024196618</v>
+        <v>0.2519863024196612</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.05860847642188649</v>
+        <v>0.05860847642188632</v>
       </c>
       <c r="E13" s="3" t="n">
         <v>0.02859587382552148</v>
@@ -740,13 +740,13 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>-0.01179209203937147</v>
+        <v>-0.01179209203937174</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>0.09479275658824517</v>
+        <v>0.09479275658824546</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>0.02522180030763105</v>
+        <v>0.02522180030763104</v>
       </c>
     </row>
     <row r="15">
@@ -761,13 +761,13 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>-0.2841259241016146</v>
+        <v>-0.284125924101614</v>
       </c>
       <c r="D15" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>0.02410164454209001</v>
+        <v>0.02410164454209</v>
       </c>
     </row>
     <row r="16">
@@ -782,7 +782,7 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.09435286896369495</v>
+        <v>0.09435286896369637</v>
       </c>
       <c r="D16" s="4" t="n">
         <v>0</v>
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.0007689419960342158</v>
+        <v>0.0007689419960341363</v>
       </c>
       <c r="D17" s="4" t="n">
         <v>0</v>
@@ -824,13 +824,13 @@
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>-0.03759225984500317</v>
+        <v>-0.03759225984500349</v>
       </c>
       <c r="D18" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>0.0242157664175613</v>
+        <v>0.02421576641756129</v>
       </c>
     </row>
     <row r="19">
@@ -866,7 +866,7 @@
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0.06848630567059005</v>
+        <v>0.06848630567059048</v>
       </c>
       <c r="D20" s="4" t="n">
         <v>0</v>
@@ -887,13 +887,13 @@
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>-0.0240442860275836</v>
+        <v>-0.02404428602758425</v>
       </c>
       <c r="D21" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>0.01674053967060342</v>
+        <v>0.01674053967060341</v>
       </c>
     </row>
     <row r="22">
@@ -908,13 +908,13 @@
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>-0.02334215103264055</v>
+        <v>-0.02334215103264168</v>
       </c>
       <c r="D22" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>0.01818953239116394</v>
+        <v>0.01818953239116393</v>
       </c>
     </row>
     <row r="23">
@@ -929,7 +929,7 @@
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>-0.08137390555190846</v>
+        <v>-0.08137390555190924</v>
       </c>
       <c r="D23" s="4" t="n">
         <v>0</v>
@@ -950,13 +950,13 @@
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0.06330023235538562</v>
+        <v>0.06330023235538591</v>
       </c>
       <c r="D24" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>0.01814629077046747</v>
+        <v>0.01814629077046746</v>
       </c>
     </row>
     <row r="25">
@@ -971,7 +971,7 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>-0.2062428010811654</v>
+        <v>-0.2062428010811646</v>
       </c>
       <c r="D25" s="4" t="n">
         <v>0</v>
@@ -992,7 +992,7 @@
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>-0.006797712678121078</v>
+        <v>-0.006797712678121018</v>
       </c>
       <c r="D26" s="4" t="n">
         <v>0</v>
@@ -1013,13 +1013,13 @@
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.1365541973418123</v>
+        <v>0.1365541973418122</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>0.09301203285013313</v>
+        <v>0.09301203285013318</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0.01708436741963163</v>
+        <v>0.01708436741963162</v>
       </c>
     </row>
     <row r="28">
@@ -1037,7 +1037,7 @@
         <v>-0.01116864284231199</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0.007311470137132811</v>
+        <v>0.007311470137132904</v>
       </c>
       <c r="E28" s="4" t="n">
         <v>0.01040840211363299</v>
@@ -1055,7 +1055,7 @@
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>0.05215998139903498</v>
+        <v>0.05215998139903533</v>
       </c>
       <c r="D29" s="4" t="n">
         <v>0</v>
@@ -1076,7 +1076,7 @@
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>-0.01726002055360381</v>
+        <v>-0.01726002055360384</v>
       </c>
       <c r="D30" s="4" t="n">
         <v>0</v>
@@ -1100,7 +1100,7 @@
         <v>0.1926868358561905</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>0.01601348061247179</v>
+        <v>0.01601348061247147</v>
       </c>
       <c r="E31" s="2" t="n">
         <v>0.02515167294869036</v>
@@ -1118,13 +1118,13 @@
         </is>
       </c>
       <c r="C32" s="3" t="n">
-        <v>0.2151128406349921</v>
+        <v>0.2151128406349918</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>0.1673455417214122</v>
+        <v>0.1673455417214127</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>0.02810971183941772</v>
+        <v>0.02810971183941771</v>
       </c>
     </row>
     <row r="33">
@@ -1139,10 +1139,10 @@
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>0.001511207032136488</v>
+        <v>0.001511207032136582</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>0.02887575803216495</v>
+        <v>0.02887575803216463</v>
       </c>
       <c r="E33" s="2" t="n">
         <v>0.02016895723916241</v>
@@ -1160,13 +1160,13 @@
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>-0.1346794428373754</v>
+        <v>-0.1346794428373752</v>
       </c>
       <c r="D34" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>0.02151334088076434</v>
+        <v>0.02151334088076433</v>
       </c>
     </row>
     <row r="35">
@@ -1181,7 +1181,7 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>-0.3233270062072678</v>
+        <v>-0.3233270062072676</v>
       </c>
       <c r="D35" s="4" t="n">
         <v>0</v>
@@ -1202,7 +1202,7 @@
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>0.01973104286682697</v>
+        <v>0.0197310428668263</v>
       </c>
       <c r="D36" s="4" t="n">
         <v>0</v>
@@ -1223,13 +1223,13 @@
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>0.1029055949777112</v>
+        <v>0.1029055949777116</v>
       </c>
       <c r="D37" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>0.01331132128527847</v>
+        <v>0.01331132128527845</v>
       </c>
     </row>
     <row r="38">
@@ -1244,13 +1244,13 @@
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>0.01330084952545615</v>
+        <v>0.01330084952545735</v>
       </c>
       <c r="D38" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>0.01168035402227889</v>
+        <v>0.01168035402227888</v>
       </c>
     </row>
     <row r="39">
@@ -1265,7 +1265,7 @@
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>-0.04160458393939195</v>
+        <v>-0.04160458393939193</v>
       </c>
       <c r="D39" s="4" t="n">
         <v>0</v>
@@ -1286,7 +1286,7 @@
         </is>
       </c>
       <c r="C40" s="3" t="n">
-        <v>0.2598542242759588</v>
+        <v>0.2598542242759572</v>
       </c>
       <c r="D40" s="4" t="n">
         <v>0</v>
@@ -1307,7 +1307,7 @@
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>-0.03297823142062024</v>
+        <v>-0.03297823142062051</v>
       </c>
       <c r="D41" s="4" t="n">
         <v>0</v>
@@ -1328,7 +1328,7 @@
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>0.07770628389295664</v>
+        <v>0.07770628389295625</v>
       </c>
       <c r="D42" s="4" t="n">
         <v>0</v>
@@ -1349,13 +1349,13 @@
         </is>
       </c>
       <c r="C43" s="2" t="n">
-        <v>-0.05282204900471407</v>
+        <v>-0.05282204900471336</v>
       </c>
       <c r="D43" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>0.0260423558958795</v>
+        <v>0.02604235589587949</v>
       </c>
     </row>
     <row r="44">
@@ -1370,7 +1370,7 @@
         </is>
       </c>
       <c r="C44" s="2" t="n">
-        <v>0.005971225783344755</v>
+        <v>0.005971225783343637</v>
       </c>
       <c r="D44" s="4" t="n">
         <v>0</v>
@@ -1391,13 +1391,13 @@
         </is>
       </c>
       <c r="C45" s="2" t="n">
-        <v>0.1385553075063062</v>
+        <v>0.1385553075063066</v>
       </c>
       <c r="D45" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>0.02465207344649824</v>
+        <v>0.02465207344649823</v>
       </c>
     </row>
     <row r="46">
@@ -1412,7 +1412,7 @@
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>-0.1655194207655397</v>
+        <v>-0.1655194207655403</v>
       </c>
       <c r="D46" s="4" t="n">
         <v>0</v>
@@ -1433,13 +1433,13 @@
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>-0.03989232843065867</v>
+        <v>-0.03989232843065699</v>
       </c>
       <c r="D47" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>0.02452218309137687</v>
+        <v>0.02452218309137686</v>
       </c>
     </row>
     <row r="48">
@@ -1454,13 +1454,13 @@
         </is>
       </c>
       <c r="C48" s="3" t="n">
-        <v>0.2299999090504479</v>
+        <v>0.2299999090504482</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>0.1366872182297593</v>
+        <v>0.1366872182297591</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>0.02786037423599331</v>
+        <v>0.0278603742359933</v>
       </c>
     </row>
     <row r="49">
@@ -1475,7 +1475,7 @@
         </is>
       </c>
       <c r="C49" s="2" t="n">
-        <v>-0.04468174767070432</v>
+        <v>-0.04468174767070498</v>
       </c>
       <c r="D49" s="4" t="n">
         <v>0</v>
@@ -1496,7 +1496,7 @@
         </is>
       </c>
       <c r="C50" s="2" t="n">
-        <v>-0.003120226308440276</v>
+        <v>-0.003120226308440688</v>
       </c>
       <c r="D50" s="4" t="n">
         <v>0</v>
@@ -1513,13 +1513,13 @@
         </is>
       </c>
       <c r="C51" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" s="6" t="n">
         <v>0.9999999999999998</v>
-      </c>
-      <c r="D51" s="6" t="n">
-        <v>0.9999999999999998</v>
-      </c>
-      <c r="E51" s="6" t="n">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>